<commit_message>
Capture complete PDF snapshots and remove whiteout geometry
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Re552d66c56b446bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R2606efef7ad94685"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,9 +23,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Escape must always fully clear selection and exit whatever edit/tool sub-state you're in, in one press, regardless of how deep the current mode is nested (81, 92)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Fix: it's possible to get permanently stuck inside a tool (e.g. right after placing a callout's arrow) with no way out — Escape doesn't help and no other tool can be switched to (82, 110)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">**(reported again, amended)** Audit and repair cursor state throughout the app. The cursor must revert as a gesture ends and must never remain as a four-way move cursor after rectangle resizing or another completed interaction. Use a context-appropriate affordance for each action: resize arrows for resize handles, a control-point-plus cursor when Shift can add a point, a control-point-minus cursor when Shift can delete one, and a curve/arc cursor when Ctrl can round a point or convert a line segment to an arc. Exercise these paths with real pointer movement, modifiers and cancellation so the cursor cannot become stuck (76, 110). **Amended 2026-09-07**: the table row/column cursor is gone with the tables.</x:t>
@@ -616,442 +613,442 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="30">
+    <x:row r="6" ht="56" customHeight="1">
       <x:c r="A6" s="2"/>
-      <x:c r="B6" s="3" t="s">
-        <x:v>5</x:v>
+      <x:c r="B6" s="3" t="str">
+        <x:v>Fix tool states that prevent cancellation or switching tools, including after placing a callout arrow. Abandon stale callout anchors and held toolset payloads when changing tools. A callout-switching defect was reproduced and repaired on 2026-09-12; the reported Escape-resistant lockup still needs a reproducing sequence (82, 110)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="90">
       <x:c r="A7" s="2"/>
       <x:c r="B7" s="3" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="30">
       <x:c r="A8" s="2"/>
       <x:c r="B8" s="3" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="45">
       <x:c r="A9" s="2"/>
       <x:c r="B9" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60">
       <x:c r="A10" s="2"/>
       <x:c r="B10" s="3" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="45">
       <x:c r="A11" s="2"/>
       <x:c r="B11" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="30">
       <x:c r="A12" s="2"/>
       <x:c r="B12" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="45">
       <x:c r="A13" s="2"/>
       <x:c r="B13" s="3" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45">
       <x:c r="A14" s="2"/>
       <x:c r="B14" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="90">
       <x:c r="A15" s="2"/>
       <x:c r="B15" s="3" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="2"/>
       <x:c r="B16" s="3" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45">
       <x:c r="A17" s="2"/>
       <x:c r="B17" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30">
       <x:c r="A18" s="2"/>
       <x:c r="B18" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="75">
       <x:c r="A19" s="2"/>
       <x:c r="B19" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="45">
       <x:c r="A21" s="2"/>
       <x:c r="B21" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="30">
       <x:c r="A22" s="2"/>
       <x:c r="B22" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2"/>
       <x:c r="B23" s="3" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="90">
       <x:c r="A24" s="2"/>
       <x:c r="B24" s="3" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="45">
       <x:c r="A25" s="2"/>
       <x:c r="B25" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="45">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="3" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30">
       <x:c r="A27" s="2"/>
       <x:c r="B27" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="45">
       <x:c r="A28" s="2"/>
       <x:c r="B28" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="30">
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="3" t="s">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="30">
       <x:c r="A30" s="2"/>
       <x:c r="B30" s="3" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="30">
       <x:c r="A31" s="2"/>
       <x:c r="B31" s="3" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="30">
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="3" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="2"/>
       <x:c r="B33" s="3" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="3" t="s">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="45">
       <x:c r="A36" s="2"/>
       <x:c r="B36" s="3" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="30">
       <x:c r="A37" s="2"/>
       <x:c r="B37" s="3" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="30">
       <x:c r="A38" s="2"/>
       <x:c r="B38" s="3" t="s">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="45">
       <x:c r="A39" s="2"/>
       <x:c r="B39" s="3" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="30">
       <x:c r="A40" s="2"/>
       <x:c r="B40" s="3" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2"/>
       <x:c r="B41" s="3" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2"/>
       <x:c r="B42" s="3" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="45">
       <x:c r="A43" s="2"/>
       <x:c r="B43" s="3" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="75">
       <x:c r="A44" s="2"/>
       <x:c r="B44" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="90">
       <x:c r="A45" s="2"/>
       <x:c r="B45" s="3" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="60">
       <x:c r="A46" s="2"/>
       <x:c r="B46" s="3" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="60">
       <x:c r="A47" s="2"/>
       <x:c r="B47" s="3" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="45">
       <x:c r="A48" s="2"/>
       <x:c r="B48" s="3" t="s">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="30">
       <x:c r="A49" s="2"/>
       <x:c r="B49" s="3" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="90">
       <x:c r="A50" s="2"/>
       <x:c r="B50" s="3" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="30">
       <x:c r="A51" s="2"/>
       <x:c r="B51" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="2"/>
       <x:c r="B52" s="3" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2"/>
       <x:c r="B53" s="3" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="30">
       <x:c r="A54" s="2"/>
       <x:c r="B54" s="3" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="30">
       <x:c r="A55" s="2"/>
       <x:c r="B55" s="3" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="2"/>
       <x:c r="B56" s="3" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="30">
       <x:c r="A57" s="2"/>
       <x:c r="B57" s="3" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="30">
       <x:c r="A58" s="2"/>
       <x:c r="B58" s="3" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="30">
       <x:c r="A59" s="2"/>
       <x:c r="B59" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="90">
       <x:c r="A60" s="2"/>
       <x:c r="B60" s="3" t="s">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="30">
       <x:c r="A61" s="2"/>
       <x:c r="B61" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2"/>
       <x:c r="B62" s="3" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="30">
       <x:c r="A63" s="2"/>
       <x:c r="B63" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="45">
       <x:c r="A64" s="2"/>
       <x:c r="B64" s="3" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="60">
       <x:c r="A65" s="2"/>
       <x:c r="B65" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="30">
       <x:c r="A66" s="2"/>
       <x:c r="B66" s="3" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="30">
       <x:c r="A67" s="2"/>
       <x:c r="B67" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="2"/>
       <x:c r="B68" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="2"/>
       <x:c r="B69" s="3" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="2"/>
       <x:c r="B70" s="3" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="45">
       <x:c r="A71" s="2"/>
       <x:c r="B71" s="3" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="45">
       <x:c r="A72" s="2"/>
       <x:c r="B72" s="3" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="45">
       <x:c r="A73" s="2"/>
       <x:c r="B73" s="3" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="30">
       <x:c r="A74" s="2"/>
       <x:c r="B74" s="3" t="s">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="45">
       <x:c r="A75" s="2"/>
       <x:c r="B75" s="3" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="45">
       <x:c r="A76" s="2"/>
       <x:c r="B76" s="3" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="60">
       <x:c r="A77" s="2"/>
       <x:c r="B77" s="3" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="60">
       <x:c r="A78" s="2"/>
       <x:c r="B78" s="3" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="56" customHeight="1">
@@ -1063,37 +1060,37 @@
     <x:row r="80" ht="45">
       <x:c r="A80" s="2"/>
       <x:c r="B80" s="3" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="75">
       <x:c r="A81" s="2"/>
       <x:c r="B81" s="3" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="120">
       <x:c r="A82" s="2"/>
       <x:c r="B82" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="45">
       <x:c r="A83" s="2"/>
       <x:c r="B83" s="3" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="60">
       <x:c r="A84" s="2"/>
       <x:c r="B84" s="3" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="60">
       <x:c r="A85" s="2"/>
       <x:c r="B85" s="3" t="s">
-        <x:v>83</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="56" customHeight="1">
@@ -1110,87 +1107,87 @@
     </x:row>
     <x:row r="88" ht="60">
       <x:c r="B88" s="3" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="30">
       <x:c r="B89" s="3" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="30">
       <x:c r="B90" s="3" t="s">
-        <x:v>86</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="60">
       <x:c r="B91" s="3" t="s">
-        <x:v>87</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="30">
       <x:c r="B92" s="3" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="30">
       <x:c r="B93" s="3" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="30">
       <x:c r="B94" s="3" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="30">
       <x:c r="B95" s="3" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="30">
       <x:c r="B96" s="3" t="s">
-        <x:v>92</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="30">
       <x:c r="B97" s="3" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="45">
       <x:c r="B98" s="3" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="30">
       <x:c r="B99" s="3" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="30">
       <x:c r="B100" s="3" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="45">
       <x:c r="B101" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="30">
       <x:c r="B102" s="3" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="30">
       <x:c r="B103" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="30">
       <x:c r="B104" s="3" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="45" customHeight="1">
@@ -1205,10 +1202,10 @@
         <x:v>Keep PDF linework sharp when zoomed out, including on high-density displays; replace temporary preview imagery with correctly resolved tiles.</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="56" customHeight="1">
+    <x:row r="107" ht="72" customHeight="1">
       <x:c r="A107"/>
       <x:c r="B107" s="4" t="str">
-        <x:v>Repair PDF snapshots so repeated capture and paste reliably include the source PDF's vector linework. Exclude paper/background fills and page background colours, and include text markups only when explicitly selected. Recolouring must remain undoable and must not change other snapshot copies that share the original recording.</x:v>
+        <x:v>Repair PDF snapshots so repeated capture and paste reliably include the source PDF's vector linework, font outlines and embedded/scanned images. Exclude paper/background fills and page background colours, and include text markups only when explicitly selected. Preserve independent PDF stroke/fill opacity. Recolouring must remain undoable and must not change other snapshot copies that share the original recording.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="45" customHeight="1">
@@ -1217,10 +1214,10 @@
         <x:v>Add adjustable hatch scale in the style toolbar and Properties panel; preserve it through copy, undo, save and PDF export.</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="45" customHeight="1">
+    <x:row r="109" ht="56" customHeight="1">
       <x:c r="A109"/>
       <x:c r="B109" s="4" t="str">
-        <x:v>Add a Whiteout tool to remove flattened PDF linework within a selected page region, with undo and correct saved/exported results.</x:v>
+        <x:v>Add a Whiteout tool that removes flattened PDF artwork and scanned pixels within a selected page region rather than merely hiding them with a clip. Preserve surviving artwork and live annotations, with undo and correct saved/exported results. Preserve searchable text outside the erased region; Whiteout is not secure redaction.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="45" customHeight="1">

</xml_diff>